<commit_message>
Update memories page series filter, remove empty mobile card, and clean UI
</commit_message>
<xml_diff>
--- a/public/fcl-series-data.xlsx
+++ b/public/fcl-series-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHL_Procurement\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEB DEVELOPER\FCL Website\Web Site Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -57,9 +57,6 @@
     <t>Golam Mohammad Manik</t>
   </si>
   <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ১ )</t>
-  </si>
-  <si>
     <t>সাবেক চেয়ারম্যান এফসিএলের ক্রিকেটকে আরও জনপ্রিয় করতে লালু ও কালু নামে দুই রোবট ক্রিকেটার তৈরি করেন। দেশসেরা কোচ আরিফ জিয়াদ তাদের প্রশিক্ষণ দিয়ে দুর্দান্ত ক্রিকেটার বানান। তাদের জনপ্রিয়তার পর WOW TV-এর উপস্থাপক তোফায়েল সাহেব আরিফ জিয়াদের বিশেষ সাক্ষাৎকার নেওয়ার সিদ্ধান্ত নেন।</t>
   </si>
   <si>
@@ -70,17 +67,11 @@
 এবার সাক্ষাৎকার দিতে ওয়াও টিভিতে হাজির আরিফ জিয়াদ ......</t>
   </si>
   <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ২ )</t>
-  </si>
-  <si>
     <t>WOW TV-এর সাক্ষাৎকারের জন্য আরিফ জিয়াদ অপেক্ষা করছেন। অন্যদিকে তোফায়েল সাহেব একটি অচেনা নম্বরের রহস্যময় ফোন পান, যেখানে ভয়ংকর হাসি, হুমকি এবং কিডন্যাপের সতর্কবার্তা দেওয়া হয়।</t>
   </si>
   <si>
     <t>আরিফ জিয়াদ রোবটের বিষয়ে সাক্ষাৎকার দেয়ার জন্য অনেক আগ্রহ নিয়ে ওয়াও টিভির ওয়েটিং রুমে বসে আছেন। ১০.৩০ টায় সাক্ষাৎকার নেওয়ার কথা থাকলেও উনি ৯.৩০ মিনিট থেকে ব্যাকুল হয়ে বসে আছেন। এদিকে তোফায়েল সাহেব তখনও বাসা থেকেই আসেননি। অফিসের উদ্দেশ্যে বাসা থেকে বের হবেন এমন সময় তোফায়েল সাহেবের ফোনটা বেজে উঠে। গত কিছুদিন ধরেই অচেনা একটা নাম্বার থেকে ফোন কল পেয়ে আসছিলেন তোফায়েল সাহেব। অপর প্রান্ত থেকে কোন এক ভয়ংকর হাসির আওয়াজ আসতে থাকে। কোন কথা না বলা সেই ফোন কল আসলেই তোফায়েল সাহেবের ভিতরটা কেমন যেনো দুমড়ে মুচড়ে উঠে।
 আজও সেই অচেনা নাম্বারের ফোন কলে ভিতরটা একেবারে শুকিয়ে গেছে তোফায়েল সাহেবের। কিন্তু আজকে হাসিতেই থেমে নেই কর্কট আওয়াজে কিছু একটা বলছিলো অপর প্রান্ত থেকে, কিন্তু ঠিকভাবে বুঝতে পারছে না তোফায়েল সাহেব। অস্পষ্ট ভাষায় কিছু একটা থেকে দূরে থাকতে বলা হচ্ছে। কথা না শুনলে কিডনাপ করার হুমকি দেয়া হয়েছে। সব ভুলে তোফায়েল সাহেব অফিসের পথে রওয়ানা হয়েছেন। এদিকে আরিফ জিয়াদ সাহেব বসে বসে তার মনে মনে সাক্ষাৎকার দেয়ার কথা গুলো সাজিয়ে নিচ্ছেন।</t>
-  </si>
-  <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ৩ )</t>
   </si>
   <si>
     <t>সাদরুল আনাম ফোন করে আরিফ জিয়াদকে সাক্ষাৎকার বাতিল করতে বলেন, কারণ রোবট সম্পর্কে মিডিয়ায় কথা বলার অধিকার তিনি শুধু নিজের জন্য রেখেছেন। কথোপকথনে সাদরুলের অস্বাভাবিক আচরণে আরিফের মনে রহস্যের সন্দেহ তৈরি হয়।</t>
@@ -99,9 +90,6 @@
 নাকি এর পেছনে অন্য কোন রহস্য লুকিয়ে আছে।
 ভাবতে ভাবতেই ভাবনার রাজ্য হারিয়ে গেলেন আরিফ জিয়াদ।
 এদিকে অফিসে ইন করলেন তোফায়েল সাহেব। কিছুক্ষণের মধ্যেই শুরু হওয়ার কথা লালু কালুর সেই বিশেষ সাক্ষাৎকার।</t>
-  </si>
-  <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ৪ )</t>
   </si>
   <si>
     <t>তোফায়েল সাহেব আরিফ জিয়াদের সাক্ষাৎকার শুরু করতে গিয়ে জানতে পারেন যে আরিফ নিখোঁজ। সাদরুল আনামকেও ফোনে পাওয়া যাচ্ছে না। পরে এক অচেনা ব্যক্তি নিজেকে নেতা পরিচয় দিয়ে জানায়, সাদরুল তার কাছে বন্দি।</t>
@@ -125,9 +113,6 @@
 _ কিন্তু সাদরুল স্যারের কি হয়েছে?
 _ বুঝো না কি হয়েছে? হাহ হা হা সাদরুল সাব এখন আমার কাছে বন্দি। কিডনাপ করছি তোমাগো সাদরুল স্যারেরে। ঐ বেটা ফোন রাখ। ধমক দিয়ে ফোন কেটে দিলো।
 অন্যদিকে কোথায় আছেন গল্পের অন্যতম চরিত্র আরিফ জিয়াদ সাহেব?</t>
-  </si>
-  <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ৫ )</t>
   </si>
   <si>
     <t>তোফায়েল সাহেব পুলিশকে জানান যে সাদরুল সাহেবকে কিডন্যাপ করা হয়েছে। পুলিশ লোকেশন ট্র্যাক করে এবং উদ্ধার অভিযানের প্রস্তুতি নেয়। এদিকে আরিফ জিয়াদ রহস্যের সমাধান করার সিদ্ধান্ত নেন।</t>
@@ -152,9 +137,6 @@
 একটু পর এফসিএলপুর মডেল থানার ওসি এসএইচ শান্ত তার টিম নিয়ে সাদরুল সাহেবকে উদ্ধারের জন্য বেরিয়ে যাবেন।
 ওসি এসএইচ শান্ত কি পারবে সাদরুল সাহেব কে
 উদ্ধার করে এফসিএলপুর' কে শান্ত করতে?</t>
-  </si>
-  <si>
-    <t>রোবটের নাম লালু কালু ( Part - 06 )</t>
   </si>
   <si>
     <t>পুলিশের উদ্ধার অভিযান নিয়ে ওসি এসএইচ শান্ত ও এসআই আকাশের মধ্যে মতবিরোধ হয়। এদিকে নেতা সাদরুলকে বন্দি করে রোবট তৈরির ফর্মুলা দাবি করে এবং সাত দিনের সময় দেয়।</t>
@@ -195,9 +177,6 @@
 অন্যদিকে আরিফ জিয়াদ ও খবর পেয়ে গেছেন সাদরুল সাহেবের কিডন্যাপড হবার বিষয়টা। এবার আরিফ জিয়াদ কি সিদ্ধান্ত নিবেন? অভিযানে যাবেন? যদি তাই যাই আরিফ জিয়াদ কি পারবে চেয়ারম্যান সাদরুল কে রক্ষা করতে?</t>
   </si>
   <si>
-    <t>রোবটের নাম লালু কালু ( পার্ট - ৭ )</t>
-  </si>
-  <si>
     <t>সাদরুলের কিডন্যাপের পর আরিফ জিয়াদ তাকে উদ্ধারের সিদ্ধান্ত নেন। লালু-কালুর গোপন GPS ও ব্যাকডোর কোড ব্যবহার করে তিনি তাদের অবস্থান শনাক্ত করেন এবং পরিত্যক্ত গুদাম এলাকায় রওনা হন। সামনে অপেক্ষা করছে জুম্মন কশাই ও রহস্যময় নেতার বাহিনীর সঙ্গে সংঘর্ষের সম্ভাবনা।</t>
   </si>
   <si>
@@ -212,6 +191,27 @@
   </si>
   <si>
     <t>Running</t>
+  </si>
+  <si>
+    <t>(পার্ট - ১)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ২)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ৩)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ৪)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ৫)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ৭)</t>
+  </si>
+  <si>
+    <t>(পার্ট - ৬)</t>
   </si>
 </sst>
 </file>
@@ -646,20 +646,20 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E2" s="5">
         <v>2021</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -673,20 +673,20 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E3" s="5">
         <v>2021</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -700,20 +700,20 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E4" s="5">
         <v>2021</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="3" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -727,20 +727,20 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E5" s="5">
         <v>2021</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -754,20 +754,20 @@
         <v>5</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E6" s="5">
         <v>2021</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -781,20 +781,20 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E7" s="5">
         <v>2021</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="7" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -808,20 +808,20 @@
         <v>7</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E8" s="5">
         <v>2026</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="5" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix series episode accordion toggle and layout in memories page
</commit_message>
<xml_diff>
--- a/public/fcl-series-data.xlsx
+++ b/public/fcl-series-data.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>series_name</t>
   </si>
@@ -191,27 +191,6 @@
   </si>
   <si>
     <t>Running</t>
-  </si>
-  <si>
-    <t>(পার্ট - ১)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ২)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ৩)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ৪)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ৫)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ৭)</t>
-  </si>
-  <si>
-    <t>(পার্ট - ৬)</t>
   </si>
 </sst>
 </file>
@@ -601,7 +580,7 @@
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="70" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="100" customWidth="1"/>
   </cols>
@@ -646,14 +625,12 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E2" s="5">
         <v>2021</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="4" t="s">
         <v>25</v>
@@ -673,14 +650,12 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E3" s="5">
         <v>2021</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="4" t="s">
         <v>25</v>
@@ -700,14 +675,12 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E4" s="5">
         <v>2021</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="4" t="s">
         <v>25</v>
@@ -727,14 +700,12 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5">
         <v>2021</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="4" t="s">
         <v>25</v>
@@ -754,14 +725,12 @@
         <v>5</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E6" s="5">
         <v>2021</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="4" t="s">
         <v>25</v>
@@ -781,14 +750,12 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E7" s="5">
         <v>2021</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="4" t="s">
         <v>25</v>
@@ -808,14 +775,12 @@
         <v>7</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E8" s="5">
         <v>2026</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>23</v>
-      </c>
+      <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="5" t="s">
         <v>25</v>

</xml_diff>